<commit_message>
feat(dashboard): revert Prev label, add real evaluation-date Open column
Signal List Performance keeps "Prev" (signal session's close) as the W/L
reference, and adds a separate "Open" column showing the evaluation
session's actual open price (informational, not used in the W/L calc).
Backfills Open for historical rows where local raw OHLC still covers the
eval date; rows outside that window are left blank rather than guessed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/performance/daily/signal_list_2026-05-19.xlsx
+++ b/data/performance/daily/signal_list_2026-05-19.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -459,12 +459,13 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,45 +495,50 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Percentage High</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Percentage Close</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>W/L High</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>W/L Close</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Eval Date</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -553,33 +559,36 @@
         <v>2630</v>
       </c>
       <c r="D5" t="n">
+        <v>2670</v>
+      </c>
+      <c r="E5" t="n">
         <v>2580</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>2670</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>1.52</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>-1.9</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -600,33 +609,36 @@
         <v>780</v>
       </c>
       <c r="D6" t="n">
+        <v>780</v>
+      </c>
+      <c r="E6" t="n">
         <v>765</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>790</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="G6" s="4" t="n">
         <v>1.28</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>-1.92</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -647,33 +659,36 @@
         <v>2310</v>
       </c>
       <c r="D7" t="n">
+        <v>2320</v>
+      </c>
+      <c r="E7" t="n">
         <v>2240</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>2460</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="G7" s="4" t="n">
         <v>6.49</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>-3.03</v>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -694,33 +709,36 @@
         <v>342</v>
       </c>
       <c r="D8" t="n">
+        <v>344</v>
+      </c>
+      <c r="E8" t="n">
         <v>338</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>350</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="G8" s="4" t="n">
         <v>2.34</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>-1.17</v>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -741,33 +759,36 @@
         <v>1600</v>
       </c>
       <c r="D9" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E9" t="n">
         <v>1590</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>1600</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="G9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>-0.62</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -788,33 +809,36 @@
         <v>154</v>
       </c>
       <c r="D10" t="n">
+        <v>154</v>
+      </c>
+      <c r="E10" t="n">
         <v>151</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>156</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="G10" s="4" t="n">
         <v>1.3</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>-1.95</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -838,30 +862,33 @@
         <v>2380</v>
       </c>
       <c r="E11" t="n">
+        <v>2380</v>
+      </c>
+      <c r="F11" t="n">
         <v>2390</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="G11" s="4" t="n">
         <v>0.42</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -882,33 +909,36 @@
         <v>1200</v>
       </c>
       <c r="D12" t="n">
+        <v>1215</v>
+      </c>
+      <c r="E12" t="n">
         <v>1175</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>1225</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>2.08</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>-2.08</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -929,33 +959,36 @@
         <v>2890</v>
       </c>
       <c r="D13" t="n">
+        <v>2600</v>
+      </c>
+      <c r="E13" t="n">
         <v>3130</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>3600</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="G13" s="4" t="n">
         <v>24.57</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -976,33 +1009,36 @@
         <v>1485</v>
       </c>
       <c r="D14" t="n">
+        <v>1485</v>
+      </c>
+      <c r="E14" t="n">
         <v>1480</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>1505</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>1.35</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>-0.34</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1023,33 +1059,36 @@
         <v>5925</v>
       </c>
       <c r="D15" t="n">
+        <v>5900</v>
+      </c>
+      <c r="E15" t="n">
         <v>5925</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>6125</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="G15" s="4" t="n">
         <v>3.38</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1070,33 +1109,36 @@
         <v>1005</v>
       </c>
       <c r="D16" t="n">
+        <v>1010</v>
+      </c>
+      <c r="E16" t="n">
         <v>995</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>1010</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>-1</v>
       </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1117,33 +1159,36 @@
         <v>1720</v>
       </c>
       <c r="D17" t="n">
+        <v>1725</v>
+      </c>
+      <c r="E17" t="n">
         <v>1710</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>1730</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>0.58</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>-0.58</v>
       </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1164,33 +1209,36 @@
         <v>71</v>
       </c>
       <c r="D18" t="n">
+        <v>71</v>
+      </c>
+      <c r="E18" t="n">
         <v>69</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>73</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="G18" s="4" t="n">
         <v>2.82</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>-2.82</v>
       </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1211,33 +1259,36 @@
         <v>775</v>
       </c>
       <c r="D19" t="n">
+        <v>775</v>
+      </c>
+      <c r="E19" t="n">
         <v>760</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>775</v>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="G19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="4" t="n">
+      <c r="H19" s="4" t="n">
         <v>-1.94</v>
       </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1258,33 +1309,36 @@
         <v>2670</v>
       </c>
       <c r="D20" t="n">
+        <v>2680</v>
+      </c>
+      <c r="E20" t="n">
         <v>2600</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>2720</v>
       </c>
-      <c r="F20" s="4" t="n">
+      <c r="G20" s="4" t="n">
         <v>1.87</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="H20" s="4" t="n">
         <v>-2.62</v>
       </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1305,33 +1359,36 @@
         <v>850</v>
       </c>
       <c r="D21" t="n">
+        <v>761.73</v>
+      </c>
+      <c r="E21" t="n">
         <v>735</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>761.73</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="G21" s="4" t="n">
         <v>-10.39</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="H21" s="4" t="n">
         <v>-13.53</v>
       </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1352,33 +1409,36 @@
         <v>6575</v>
       </c>
       <c r="D22" t="n">
+        <v>6750</v>
+      </c>
+      <c r="E22" t="n">
         <v>5950</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>6775</v>
       </c>
-      <c r="F22" s="4" t="n">
+      <c r="G22" s="4" t="n">
         <v>3.04</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="H22" s="4" t="n">
         <v>-9.51</v>
       </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1399,33 +1459,36 @@
         <v>550</v>
       </c>
       <c r="D23" t="n">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="E23" t="n">
         <v>555</v>
       </c>
-      <c r="F23" s="4" t="n">
-        <v>0.91</v>
+      <c r="F23" t="n">
+        <v>555</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>0.91</v>
       </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
+      <c r="H23" s="4" t="n">
+        <v>0.91</v>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1446,33 +1509,36 @@
         <v>1800</v>
       </c>
       <c r="D24" t="n">
+        <v>1765</v>
+      </c>
+      <c r="E24" t="n">
         <v>1770</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>1795</v>
       </c>
-      <c r="F24" s="4" t="n">
+      <c r="G24" s="4" t="n">
         <v>-0.28</v>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="H24" s="4" t="n">
         <v>-1.67</v>
       </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1493,33 +1559,36 @@
         <v>945</v>
       </c>
       <c r="D25" t="n">
+        <v>950</v>
+      </c>
+      <c r="E25" t="n">
         <v>855</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>950</v>
       </c>
-      <c r="F25" s="4" t="n">
+      <c r="G25" s="4" t="n">
         <v>0.53</v>
       </c>
-      <c r="G25" s="4" t="n">
+      <c r="H25" s="4" t="n">
         <v>-9.52</v>
       </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1540,33 +1609,36 @@
         <v>240</v>
       </c>
       <c r="D26" t="n">
+        <v>252</v>
+      </c>
+      <c r="E26" t="n">
         <v>234</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>252</v>
       </c>
-      <c r="F26" s="4" t="n">
+      <c r="G26" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="G26" s="4" t="n">
+      <c r="H26" s="4" t="n">
         <v>-2.5</v>
       </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1587,33 +1659,36 @@
         <v>224</v>
       </c>
       <c r="D27" t="n">
+        <v>226</v>
+      </c>
+      <c r="E27" t="n">
         <v>218</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>234</v>
       </c>
-      <c r="F27" s="4" t="n">
+      <c r="G27" s="4" t="n">
         <v>4.46</v>
       </c>
-      <c r="G27" s="4" t="n">
+      <c r="H27" s="4" t="n">
         <v>-2.68</v>
       </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1634,33 +1709,36 @@
         <v>420</v>
       </c>
       <c r="D28" t="n">
+        <v>422</v>
+      </c>
+      <c r="E28" t="n">
         <v>426</v>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>434</v>
       </c>
-      <c r="F28" s="4" t="n">
+      <c r="G28" s="4" t="n">
         <v>3.33</v>
       </c>
-      <c r="G28" s="4" t="n">
+      <c r="H28" s="4" t="n">
         <v>1.43</v>
       </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1681,33 +1759,36 @@
         <v>157</v>
       </c>
       <c r="D29" t="n">
+        <v>157</v>
+      </c>
+      <c r="E29" t="n">
         <v>156</v>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>159</v>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="G29" s="4" t="n">
         <v>1.27</v>
       </c>
-      <c r="G29" s="4" t="n">
+      <c r="H29" s="4" t="n">
         <v>-0.64</v>
       </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1728,33 +1809,36 @@
         <v>985</v>
       </c>
       <c r="D30" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E30" t="n">
         <v>1010</v>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>1030</v>
       </c>
-      <c r="F30" s="4" t="n">
+      <c r="G30" s="4" t="n">
         <v>4.57</v>
       </c>
-      <c r="G30" s="4" t="n">
+      <c r="H30" s="4" t="n">
         <v>2.54</v>
       </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1775,33 +1859,36 @@
         <v>220</v>
       </c>
       <c r="D31" t="n">
+        <v>220</v>
+      </c>
+      <c r="E31" t="n">
         <v>218</v>
       </c>
-      <c r="E31" t="n">
+      <c r="F31" t="n">
         <v>224</v>
       </c>
-      <c r="F31" s="4" t="n">
+      <c r="G31" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="G31" s="4" t="n">
+      <c r="H31" s="4" t="n">
         <v>-0.91</v>
       </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1822,33 +1909,36 @@
         <v>80</v>
       </c>
       <c r="D32" t="n">
+        <v>80</v>
+      </c>
+      <c r="E32" t="n">
         <v>73</v>
       </c>
-      <c r="E32" t="n">
+      <c r="F32" t="n">
         <v>81</v>
       </c>
-      <c r="F32" s="4" t="n">
+      <c r="G32" s="4" t="n">
         <v>1.25</v>
       </c>
-      <c r="G32" s="4" t="n">
+      <c r="H32" s="4" t="n">
         <v>-8.75</v>
       </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1869,33 +1959,36 @@
         <v>494</v>
       </c>
       <c r="D33" t="n">
+        <v>500</v>
+      </c>
+      <c r="E33" t="n">
         <v>432</v>
       </c>
-      <c r="E33" t="n">
+      <c r="F33" t="n">
         <v>500</v>
       </c>
-      <c r="F33" s="4" t="n">
+      <c r="G33" s="4" t="n">
         <v>1.21</v>
       </c>
-      <c r="G33" s="4" t="n">
+      <c r="H33" s="4" t="n">
         <v>-12.55</v>
       </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1916,33 +2009,36 @@
         <v>7125</v>
       </c>
       <c r="D34" t="n">
-        <v>7175</v>
+        <v>7125</v>
       </c>
       <c r="E34" t="n">
         <v>7175</v>
       </c>
-      <c r="F34" s="4" t="n">
-        <v>0.7</v>
+      <c r="F34" t="n">
+        <v>7175</v>
       </c>
       <c r="G34" s="4" t="n">
         <v>0.7</v>
       </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
+      <c r="H34" s="4" t="n">
+        <v>0.7</v>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -1963,33 +2059,36 @@
         <v>2460</v>
       </c>
       <c r="D35" t="n">
+        <v>2460</v>
+      </c>
+      <c r="E35" t="n">
         <v>2330</v>
       </c>
-      <c r="E35" t="n">
+      <c r="F35" t="n">
         <v>2470</v>
       </c>
-      <c r="F35" s="4" t="n">
+      <c r="G35" s="4" t="n">
         <v>0.41</v>
       </c>
-      <c r="G35" s="4" t="n">
+      <c r="H35" s="4" t="n">
         <v>-5.28</v>
       </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>evaluated</t>
         </is>
@@ -2006,7 +2105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2014,12 +2113,13 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2049,45 +2149,50 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>Prev</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Percentage High</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Percentage Close</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>W/L High</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>W/L Close</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Eval Date</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>

</xml_diff>